<commit_message>
Generalizar introduccion de la encuesta
</commit_message>
<xml_diff>
--- a/data/content/instrumento_DCE.xlsx
+++ b/data/content/instrumento_DCE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7107fc2c64664341/Documentos/tesis_dce/data/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_0D4BFA71817179448C069D406CB4DC3B973B4277" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4231A7F-7246-4C57-9FB7-41CB70DF6A2E}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_0D4BFA71817179448C069D406CB4DC3B973B4277" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28A76D9D-2A84-4D91-87E2-27B64AC84E74}"/>
   <bookViews>
-    <workbookView xWindow="5220" yWindow="3540" windowWidth="21600" windowHeight="11835" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5220" yWindow="3540" windowWidth="21600" windowHeight="11835" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -682,18 +682,12 @@
     <t>titulo</t>
   </si>
   <si>
-    <t>Encuesta sobre soluciones de inteligencia artificial para empresas del comercio minorista</t>
-  </si>
-  <si>
     <t>bienvenida_intro</t>
   </si>
   <si>
     <t>parrafo</t>
   </si>
   <si>
-    <t>Esta encuesta forma parte de una investigación académica sobre la valoración de soluciones basadas en inteligencia artificial por parte de pequeñas y medianas empresas del comercio minorista.</t>
-  </si>
-  <si>
     <t>consentimiento</t>
   </si>
   <si>
@@ -1361,6 +1355,13 @@
   </si>
   <si>
     <t>Otra actividad (distinta de las anteriores)</t>
+  </si>
+  <si>
+    <t>Encuesta sobre soluciones de inteligencia artificial para empresas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esta encuesta forma parte de una investigación académica sobre la valoración de soluciones basadas en inteligencia artificial por parte de empresas.
+</t>
   </si>
 </sst>
 </file>
@@ -1507,6 +1508,10 @@
     </a>
   </bag>
 </FeaturePropertyBags>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2422,7 +2427,7 @@
         <v>102</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D10" s="4">
         <v>1</v>
@@ -2436,7 +2441,7 @@
         <v>103</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D11" s="4">
         <v>2</v>
@@ -2450,7 +2455,7 @@
         <v>104</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="D12" s="4">
         <v>3</v>
@@ -2464,7 +2469,7 @@
         <v>105</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="D13" s="4">
         <v>4</v>
@@ -2478,7 +2483,7 @@
         <v>106</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="D14" s="4">
         <v>5</v>
@@ -3304,13 +3309,13 @@
       <c r="D2" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>218</v>
+      <c r="E2" t="s">
+        <v>443</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="42.75">
       <c r="A3" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>216</v>
@@ -3319,15 +3324,15 @@
         <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>221</v>
+        <v>444</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="42.75">
       <c r="A4" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>216</v>
@@ -3336,15 +3341,15 @@
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="42.75">
       <c r="A5" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>50</v>
@@ -3353,35 +3358,35 @@
         <v>1</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="42.75">
       <c r="A6" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C6" s="4">
         <v>1</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C7" s="4">
         <v>1</v>
@@ -3390,24 +3395,24 @@
         <v>217</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="57">
       <c r="A8" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C8" s="4">
         <v>2</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -3436,13 +3441,13 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15">
       <c r="A1" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>233</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>235</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>41</v>
@@ -3450,13 +3455,13 @@
     </row>
     <row r="2" spans="1:4" ht="42.75">
       <c r="A2" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>236</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>238</v>
       </c>
       <c r="D2" s="9">
         <v>1</v>
@@ -3464,13 +3469,13 @@
     </row>
     <row r="3" spans="1:4" ht="42.75">
       <c r="A3" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>241</v>
       </c>
       <c r="D3" s="4">
         <v>2</v>
@@ -3478,13 +3483,13 @@
     </row>
     <row r="4" spans="1:4" ht="28.5">
       <c r="A4" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>242</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>244</v>
       </c>
       <c r="D4" s="9">
         <v>3</v>
@@ -3512,16 +3517,16 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15">
       <c r="A1" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>233</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>245</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>235</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>41</v>
@@ -3530,16 +3535,16 @@
     </row>
     <row r="2" spans="1:7" ht="28.5">
       <c r="A2" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B2" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>246</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>248</v>
       </c>
       <c r="E2" s="9">
         <v>1</v>
@@ -3548,16 +3553,16 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>249</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>251</v>
       </c>
       <c r="E3" s="4">
         <v>2</v>
@@ -3565,16 +3570,16 @@
     </row>
     <row r="4" spans="1:7" ht="28.5">
       <c r="A4" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>252</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>254</v>
       </c>
       <c r="E4" s="9">
         <v>3</v>
@@ -3582,16 +3587,16 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>255</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>257</v>
       </c>
       <c r="E5" s="4">
         <v>4</v>
@@ -3599,16 +3604,16 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B6" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>258</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>260</v>
       </c>
       <c r="E6" s="9">
         <v>5</v>
@@ -3616,16 +3621,16 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>261</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>263</v>
       </c>
       <c r="E7" s="4">
         <v>6</v>
@@ -3633,16 +3638,16 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B8" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>266</v>
       </c>
       <c r="E8" s="9">
         <v>1</v>
@@ -3650,16 +3655,16 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>267</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>269</v>
       </c>
       <c r="E9" s="4">
         <v>2</v>
@@ -3667,16 +3672,16 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B10" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>270</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>272</v>
       </c>
       <c r="E10" s="9">
         <v>3</v>
@@ -3684,16 +3689,16 @@
     </row>
     <row r="11" spans="1:7" ht="28.5">
       <c r="A11" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>273</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>275</v>
       </c>
       <c r="E11" s="4">
         <v>4</v>
@@ -3701,16 +3706,16 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>276</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>278</v>
       </c>
       <c r="E12" s="9">
         <v>5</v>
@@ -3718,16 +3723,16 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>261</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>263</v>
       </c>
       <c r="E13" s="4">
         <v>6</v>
@@ -3735,16 +3740,16 @@
     </row>
     <row r="14" spans="1:7" ht="28.5">
       <c r="A14" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B14" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>279</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>280</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>281</v>
       </c>
       <c r="E14" s="9">
         <v>1</v>
@@ -3752,16 +3757,16 @@
     </row>
     <row r="15" spans="1:7" ht="28.5">
       <c r="A15" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>282</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>284</v>
       </c>
       <c r="E15" s="4">
         <v>2</v>
@@ -3769,16 +3774,16 @@
     </row>
     <row r="16" spans="1:7" ht="28.5">
       <c r="A16" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B16" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>285</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>286</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>287</v>
       </c>
       <c r="E16" s="9">
         <v>3</v>
@@ -3786,16 +3791,16 @@
     </row>
     <row r="17" spans="1:5" ht="28.5">
       <c r="A17" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E17" s="4">
         <v>4</v>
@@ -3803,16 +3808,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>261</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>263</v>
       </c>
       <c r="E18" s="9">
         <v>5</v>
@@ -3838,19 +3843,19 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15">
       <c r="A1" s="8" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>85</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>41</v>
@@ -3859,19 +3864,19 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>291</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>293</v>
       </c>
       <c r="F2" s="9">
         <v>0</v>
@@ -3880,19 +3885,19 @@
     </row>
     <row r="3" spans="1:8" ht="28.5">
       <c r="A3" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>294</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>296</v>
       </c>
       <c r="F3" s="4">
         <v>1</v>
@@ -3900,19 +3905,19 @@
     </row>
     <row r="4" spans="1:8" ht="28.5">
       <c r="A4" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C4" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>297</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>298</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>299</v>
       </c>
       <c r="F4" s="9">
         <v>2</v>
@@ -3920,19 +3925,19 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>300</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>302</v>
       </c>
       <c r="F5" s="4">
         <v>3</v>
@@ -3940,19 +3945,19 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>303</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>305</v>
       </c>
       <c r="F6" s="9">
         <v>0</v>
@@ -3960,19 +3965,19 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>306</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>308</v>
       </c>
       <c r="F7" s="4">
         <v>1</v>
@@ -3980,19 +3985,19 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>308</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>309</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>310</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>311</v>
       </c>
       <c r="F8" s="9">
         <v>2</v>
@@ -4000,19 +4005,19 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>312</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>314</v>
       </c>
       <c r="F9" s="4">
         <v>3</v>
@@ -4020,19 +4025,19 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="F10" s="9">
         <v>0</v>
@@ -4040,19 +4045,19 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>316</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>318</v>
       </c>
       <c r="F11" s="4">
         <v>1</v>
@@ -4060,19 +4065,19 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>319</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>320</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>321</v>
       </c>
       <c r="F12" s="9">
         <v>2</v>
@@ -4080,19 +4085,19 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>322</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>324</v>
       </c>
       <c r="F13" s="4">
         <v>3</v>
@@ -4100,19 +4105,19 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F14" s="9">
         <v>0</v>
@@ -4120,19 +4125,19 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="F15" s="4">
         <v>1</v>
@@ -4140,19 +4145,19 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="E16" s="9" t="s">
         <v>328</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>330</v>
       </c>
       <c r="F16" s="9">
         <v>2</v>
@@ -4160,19 +4165,19 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>331</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>333</v>
       </c>
       <c r="F17" s="4">
         <v>3</v>
@@ -4180,19 +4185,19 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>334</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>336</v>
       </c>
       <c r="F18" s="9">
         <v>1</v>
@@ -4200,19 +4205,19 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>337</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>339</v>
       </c>
       <c r="F19" s="4">
         <v>2</v>
@@ -4220,19 +4225,19 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C20" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>340</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>341</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>342</v>
       </c>
       <c r="F20" s="9">
         <v>3</v>
@@ -4240,19 +4245,19 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>343</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>344</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>345</v>
       </c>
       <c r="F21" s="4">
         <v>1</v>
@@ -4260,19 +4265,19 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C22" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>346</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>347</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>348</v>
       </c>
       <c r="F22" s="9">
         <v>2</v>
@@ -4280,19 +4285,19 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>349</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>351</v>
       </c>
       <c r="F23" s="4">
         <v>3</v>
@@ -4300,19 +4305,19 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C24" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E24" s="9" t="s">
         <v>352</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>353</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>354</v>
       </c>
       <c r="F24" s="9">
         <v>1</v>
@@ -4320,19 +4325,19 @@
     </row>
     <row r="25" spans="1:6" ht="28.5">
       <c r="A25" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>355</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>357</v>
       </c>
       <c r="F25" s="4">
         <v>2</v>
@@ -4340,19 +4345,19 @@
     </row>
     <row r="26" spans="1:6" ht="28.5">
       <c r="A26" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C26" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="E26" s="9" t="s">
         <v>358</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>359</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>360</v>
       </c>
       <c r="F26" s="9">
         <v>3</v>
@@ -4360,19 +4365,19 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>361</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>363</v>
       </c>
       <c r="F27" s="4">
         <v>0</v>
@@ -4380,19 +4385,19 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C28" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="E28" s="9" t="s">
         <v>364</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>365</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>366</v>
       </c>
       <c r="F28" s="9">
         <v>1</v>
@@ -4400,19 +4405,19 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>367</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>369</v>
       </c>
       <c r="F29" s="4">
         <v>2</v>
@@ -4420,19 +4425,19 @@
     </row>
     <row r="30" spans="1:6" ht="28.5">
       <c r="A30" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C30" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="E30" s="9" t="s">
         <v>370</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>371</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>372</v>
       </c>
       <c r="F30" s="9">
         <v>3</v>
@@ -4440,19 +4445,19 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="F31" s="4">
         <v>0</v>
@@ -4460,19 +4465,19 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="E32" s="9" t="s">
         <v>374</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>375</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>376</v>
       </c>
       <c r="F32" s="9">
         <v>1</v>
@@ -4480,19 +4485,19 @@
     </row>
     <row r="33" spans="1:6" ht="28.5">
       <c r="A33" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C33" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>377</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>379</v>
       </c>
       <c r="F33" s="4">
         <v>0</v>
@@ -4500,19 +4505,19 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="E34" s="9" t="s">
         <v>380</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>381</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>382</v>
       </c>
       <c r="F34" s="9">
         <v>1</v>
@@ -4520,19 +4525,19 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C35" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>383</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>384</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>385</v>
       </c>
       <c r="F35" s="4">
         <v>2</v>
@@ -4540,19 +4545,19 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C36" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="E36" s="9" t="s">
         <v>386</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>387</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>388</v>
       </c>
       <c r="F36" s="9">
         <v>0</v>
@@ -4560,19 +4565,19 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C37" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>389</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>391</v>
       </c>
       <c r="F37" s="4">
         <v>1</v>
@@ -4580,19 +4585,19 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C38" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="E38" s="9" t="s">
         <v>392</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>393</v>
-      </c>
-      <c r="E38" s="9" t="s">
-        <v>394</v>
       </c>
       <c r="F38" s="9">
         <v>1</v>
@@ -4600,19 +4605,19 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>395</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>397</v>
       </c>
       <c r="F39" s="4">
         <v>2</v>
@@ -4620,19 +4625,19 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C40" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="E40" s="9" t="s">
         <v>398</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>399</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>400</v>
       </c>
       <c r="F40" s="9">
         <v>3</v>
@@ -4640,19 +4645,19 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F41" s="4">
         <v>0</v>
@@ -4660,19 +4665,19 @@
     </row>
     <row r="42" spans="1:6" ht="28.5">
       <c r="A42" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C42" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="E42" s="9" t="s">
         <v>402</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>403</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>404</v>
       </c>
       <c r="F42" s="9">
         <v>1</v>
@@ -4680,19 +4685,19 @@
     </row>
     <row r="43" spans="1:6" ht="28.5">
       <c r="A43" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C43" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>405</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>407</v>
       </c>
       <c r="F43" s="4">
         <v>2</v>
@@ -4700,19 +4705,19 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="F44" s="9">
         <v>0</v>
@@ -4720,19 +4725,19 @@
     </row>
     <row r="45" spans="1:6" ht="28.5">
       <c r="A45" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C45" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>409</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>410</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>411</v>
       </c>
       <c r="F45" s="4">
         <v>1</v>
@@ -4740,19 +4745,19 @@
     </row>
     <row r="46" spans="1:6">
       <c r="A46" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C46" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="E46" s="9" t="s">
         <v>412</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>414</v>
       </c>
       <c r="F46" s="9">
         <v>2</v>
@@ -4760,19 +4765,19 @@
     </row>
     <row r="47" spans="1:6" ht="28.5">
       <c r="A47" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C47" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="E47" s="4" t="s">
         <v>415</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>417</v>
       </c>
       <c r="F47" s="4">
         <v>3</v>
@@ -4780,19 +4785,19 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F48" s="9">
         <v>0</v>
@@ -4800,19 +4805,19 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C49" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="E49" s="4" t="s">
         <v>419</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>421</v>
       </c>
       <c r="F49" s="4">
         <v>1</v>
@@ -4820,19 +4825,19 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C50" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="E50" s="9" t="s">
         <v>422</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="E50" s="9" t="s">
-        <v>424</v>
       </c>
       <c r="F50" s="9">
         <v>2</v>
@@ -4840,19 +4845,19 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C51" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="E51" s="4" t="s">
         <v>425</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>426</v>
-      </c>
-      <c r="E51" s="4" t="s">
-        <v>427</v>
       </c>
       <c r="F51" s="4">
         <v>0</v>
@@ -4860,19 +4865,19 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C52" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="E52" s="9" t="s">
         <v>428</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>429</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>430</v>
       </c>
       <c r="F52" s="9">
         <v>1</v>
@@ -4880,19 +4885,19 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B53" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C53" t="s">
+        <v>429</v>
+      </c>
+      <c r="D53" t="s">
+        <v>430</v>
+      </c>
+      <c r="E53" t="s">
         <v>431</v>
-      </c>
-      <c r="D53" t="s">
-        <v>432</v>
-      </c>
-      <c r="E53" t="s">
-        <v>433</v>
       </c>
       <c r="F53">
         <v>1</v>
@@ -4900,19 +4905,19 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B54" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C54" t="s">
+        <v>432</v>
+      </c>
+      <c r="D54" t="s">
+        <v>433</v>
+      </c>
+      <c r="E54" t="s">
         <v>434</v>
-      </c>
-      <c r="D54" t="s">
-        <v>435</v>
-      </c>
-      <c r="E54" t="s">
-        <v>436</v>
       </c>
       <c r="F54">
         <v>2</v>
@@ -4920,19 +4925,19 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B55" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C55" t="s">
+        <v>435</v>
+      </c>
+      <c r="D55" t="s">
+        <v>436</v>
+      </c>
+      <c r="E55" t="s">
         <v>437</v>
-      </c>
-      <c r="D55" t="s">
-        <v>438</v>
-      </c>
-      <c r="E55" t="s">
-        <v>439</v>
       </c>
       <c r="F55">
         <v>3</v>

</xml_diff>